<commit_message>
state: 2026-10-21 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/programs.xlsx
+++ b/out/programs.xlsx
@@ -15114,7 +15114,7 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>Already watched by pwp-careers</t>
+          <t>Already watched by pwp-events</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -15139,7 +15139,7 @@
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>Simplify's list names the U.S. Perella Weinberg Advisory Prep Program for sophomores. No ATS link found on the page.</t>
+          <t>Simplify's list names the U.S. Perella Weinberg Advisory Prep Program for sophomores. No ATS link found on the page. Correction 2026-10-20: the intern page links a tal.net board (pwpcareers.tal.net); its events feed lists the U.S. Advisory Prep Program.</t>
         </is>
       </c>
     </row>

</xml_diff>